<commit_message>
Refresh mortgage rate to current FRED 30-yr average (6.66%)
Brings the repo in sync with the rate already live in production
(data/mortgage-rate.json refresh script had updated the rate calculator
default on every listing page and property_listings.xlsx, but the
change hadn't been committed).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listings/property_listings.xlsx
+++ b/listings/property_listings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1b8a2bdd8672135/Documents/website/listings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFB1FE30-AC31-4407-84D1-73B31E2127B4}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AA45C1B-2D7A-4FB9-8B49-2C1C3FA6523F}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -711,9 +711,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -756,12 +753,6 @@
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -771,16 +762,25 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1098,22 +1098,22 @@
   <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.36328125" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" style="11" customWidth="1"/>
-    <col min="3" max="3" width="14" style="11" customWidth="1"/>
-    <col min="4" max="4" width="38" style="11" customWidth="1"/>
-    <col min="5" max="5" width="14" style="11" customWidth="1"/>
-    <col min="6" max="6" width="16" style="11" customWidth="1"/>
-    <col min="7" max="7" width="14" style="32" customWidth="1"/>
-    <col min="8" max="8" width="16" style="11" customWidth="1"/>
-    <col min="9" max="10" width="7" style="11" customWidth="1"/>
-    <col min="11" max="11" width="14" style="11" customWidth="1"/>
-    <col min="12" max="12" width="9" style="11" customWidth="1"/>
-    <col min="13" max="13" width="20" style="11" customWidth="1"/>
-    <col min="14" max="14" width="255.81640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="41.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="70.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.7265625" style="11"/>
+    <col min="1" max="1" width="36.36328125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="10" customWidth="1"/>
+    <col min="3" max="3" width="14" style="10" customWidth="1"/>
+    <col min="4" max="4" width="38" style="10" customWidth="1"/>
+    <col min="5" max="5" width="14" style="10" customWidth="1"/>
+    <col min="6" max="6" width="16" style="10" customWidth="1"/>
+    <col min="7" max="7" width="14" style="27" customWidth="1"/>
+    <col min="8" max="8" width="16" style="10" customWidth="1"/>
+    <col min="9" max="10" width="7" style="10" customWidth="1"/>
+    <col min="11" max="11" width="14" style="10" customWidth="1"/>
+    <col min="12" max="12" width="9" style="10" customWidth="1"/>
+    <col min="13" max="13" width="20" style="10" customWidth="1"/>
+    <col min="14" max="14" width="255.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="41.453125" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="70.453125" style="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1135,7 +1135,7 @@
       <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
@@ -1159,10 +1159,10 @@
       <c r="N1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="P1" s="13" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1182,10 +1182,10 @@
       <c r="E2" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="15">
         <v>359000</v>
       </c>
       <c r="H2" s="9" t="s">
@@ -1201,16 +1201,16 @@
         <v>896</v>
       </c>
       <c r="L2" s="8"/>
-      <c r="M2" s="17">
+      <c r="M2" s="16">
         <v>1961</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="N2" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="O2" s="19" t="s">
+      <c r="O2" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="P2" s="20" t="s">
+      <c r="P2" s="19" t="s">
         <v>146</v>
       </c>
     </row>
@@ -1230,10 +1230,10 @@
       <c r="E3" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="15">
         <v>375000</v>
       </c>
       <c r="H3" s="9" t="s">
@@ -1249,21 +1249,21 @@
         <v>896</v>
       </c>
       <c r="L3" s="8"/>
-      <c r="M3" s="17">
+      <c r="M3" s="16">
         <v>1961</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="17" t="s">
         <v>140</v>
       </c>
       <c r="O3" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="P3" s="20" t="s">
+      <c r="P3" s="19" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="20" t="s">
         <v>142</v>
       </c>
       <c r="B4" s="8">
@@ -1272,16 +1272,16 @@
       <c r="C4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="20" t="s">
         <v>155</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="15">
         <v>400000</v>
       </c>
       <c r="H4" s="9" t="s">
@@ -1297,293 +1297,293 @@
         <v>896</v>
       </c>
       <c r="L4" s="8"/>
-      <c r="M4" s="17">
+      <c r="M4" s="16">
         <v>1961</v>
       </c>
-      <c r="N4" s="18" t="s">
+      <c r="N4" s="17" t="s">
         <v>143</v>
       </c>
       <c r="O4" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="P4" s="20" t="s">
+      <c r="P4" s="19" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="B5" s="7">
-        <v>6797131</v>
+        <v>43</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>44</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>124</v>
+        <v>36</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>45</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="G5" s="16">
-        <v>590000</v>
+      <c r="F5" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="21">
+        <v>550000</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="8">
-        <v>3</v>
-      </c>
-      <c r="J5" s="8">
-        <v>3</v>
-      </c>
-      <c r="K5" s="8">
-        <v>1514</v>
-      </c>
-      <c r="L5" s="8">
-        <v>1</v>
-      </c>
-      <c r="M5" s="17">
+      <c r="I5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="16">
         <v>2024</v>
       </c>
-      <c r="N5" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="O5" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="P5" s="20" t="s">
-        <v>126</v>
+      <c r="N5" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="O5" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="P5" s="19" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="G6" s="22">
-        <v>590000</v>
+      <c r="F6" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="21">
+        <v>570000</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="M6" s="17">
+      <c r="M6" s="16">
         <v>2026</v>
       </c>
-      <c r="N6" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="O6" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="P6" s="20" t="s">
-        <v>120</v>
+      <c r="N6" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="P6" s="19" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>35</v>
+        <v>125</v>
+      </c>
+      <c r="B7" s="7">
+        <v>6797131</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>37</v>
+        <v>17</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>124</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="G7" s="22">
-        <v>570000</v>
+      <c r="F7" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="G7" s="15">
+        <v>590000</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="17">
-        <v>2026</v>
-      </c>
-      <c r="N7" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="O7" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="P7" s="20" t="s">
-        <v>121</v>
+      <c r="I7" s="8">
+        <v>3</v>
+      </c>
+      <c r="J7" s="8">
+        <v>3</v>
+      </c>
+      <c r="K7" s="8">
+        <v>1514</v>
+      </c>
+      <c r="L7" s="8">
+        <v>1</v>
+      </c>
+      <c r="M7" s="16">
+        <v>2024</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="O7" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="P7" s="19" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="G8" s="22">
-        <v>595000</v>
+      <c r="F8" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="G8" s="21">
+        <v>590000</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="M8" s="17">
-        <v>2024</v>
-      </c>
-      <c r="N8" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="O8" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="P8" s="20" t="s">
-        <v>122</v>
+      <c r="M8" s="16">
+        <v>2026</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="O8" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="P8" s="19" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="G9" s="22">
-        <v>550000</v>
+      <c r="F9" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="21">
+        <v>595000</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>20</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="M9" s="17">
+        <v>23</v>
+      </c>
+      <c r="M9" s="16">
         <v>2024</v>
       </c>
-      <c r="N9" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="O9" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="P9" s="20" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="78" x14ac:dyDescent="0.35">
+      <c r="N9" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="O9" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="P9" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="G10" s="22">
-        <v>640000</v>
+      <c r="F10" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" s="21">
+        <v>625000</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>21</v>
@@ -1592,48 +1592,48 @@
         <v>27</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="17">
-        <v>2024</v>
-      </c>
-      <c r="N10" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="O10" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="P10" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+      <c r="M10" s="16">
+        <v>2026</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="O10" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="P10" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="78" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" s="22">
-        <v>625000</v>
+      <c r="F11" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="G11" s="21">
+        <v>640000</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>21</v>
@@ -1642,22 +1642,22 @@
         <v>27</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="M11" s="17">
-        <v>2026</v>
-      </c>
-      <c r="N11" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="O11" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="P11" s="20" t="s">
-        <v>118</v>
+        <v>23</v>
+      </c>
+      <c r="M11" s="16">
+        <v>2024</v>
+      </c>
+      <c r="N11" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="O11" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="P11" s="19" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
@@ -1676,10 +1676,10 @@
       <c r="E12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="21">
         <v>685000</v>
       </c>
       <c r="H12" s="9" t="s">
@@ -1697,117 +1697,117 @@
       <c r="L12" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M12" s="17">
+      <c r="M12" s="16">
         <v>2026</v>
       </c>
-      <c r="N12" s="18" t="s">
+      <c r="N12" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="O12" s="17" t="s">
+      <c r="O12" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="P12" s="20" t="s">
+      <c r="P12" s="19" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="52" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>50</v>
+        <v>148</v>
+      </c>
+      <c r="B13" s="9">
+        <v>9547484</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>51</v>
+        <v>147</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="G13" s="22">
-        <v>715000</v>
+        <v>19</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="G13" s="21">
+        <v>699000</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M13" s="17">
-        <v>2026</v>
-      </c>
-      <c r="N13" s="24" t="s">
-        <v>154</v>
-      </c>
-      <c r="O13" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="P13" s="20" t="s">
-        <v>117</v>
+      <c r="M13" s="16">
+        <v>2023</v>
+      </c>
+      <c r="N13" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="O13" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="P13" s="19" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="52" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="B14" s="9">
-        <v>9547484</v>
+        <v>49</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>147</v>
+        <v>51</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>156</v>
-      </c>
-      <c r="G14" s="22">
-        <v>699000</v>
+        <v>52</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="G14" s="21">
+        <v>715000</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>20</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="L14" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M14" s="17">
-        <v>2023</v>
+      <c r="M14" s="16">
+        <v>2026</v>
       </c>
       <c r="N14" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="O14" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="P14" s="20" t="s">
-        <v>149</v>
+        <v>154</v>
+      </c>
+      <c r="O14" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="P14" s="19" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
@@ -1826,10 +1826,10 @@
       <c r="E15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="21">
         <v>830000</v>
       </c>
       <c r="H15" s="9" t="s">
@@ -1847,16 +1847,16 @@
       <c r="L15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="17">
+      <c r="M15" s="16">
         <v>2026</v>
       </c>
-      <c r="N15" s="18" t="s">
+      <c r="N15" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="O15" s="26" t="s">
+      <c r="O15" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="P15" s="20" t="s">
+      <c r="P15" s="19" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1876,10 +1876,10 @@
       <c r="E16" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="21">
         <v>850000</v>
       </c>
       <c r="H16" s="9" t="s">
@@ -1897,16 +1897,16 @@
       <c r="L16" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M16" s="17">
+      <c r="M16" s="16">
         <v>2026</v>
       </c>
-      <c r="N16" s="18" t="s">
+      <c r="N16" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="O16" s="27" t="s">
+      <c r="O16" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="20" t="s">
+      <c r="P16" s="19" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1926,10 +1926,10 @@
       <c r="E17" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="21">
         <v>1000000</v>
       </c>
       <c r="H17" s="9" t="s">
@@ -1947,16 +1947,16 @@
       <c r="L17" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="17">
+      <c r="M17" s="16">
         <v>2026</v>
       </c>
-      <c r="N17" s="23" t="s">
+      <c r="N17" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O17" s="17" t="s">
+      <c r="O17" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="P17" s="20" t="s">
+      <c r="P17" s="19" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1964,149 +1964,149 @@
       <c r="A18" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="31">
         <v>6600690</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="G18" s="30">
+      <c r="G18" s="32">
         <v>1300000</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K18" s="31">
         <v>4013</v>
       </c>
-      <c r="L18" s="10" t="s">
+      <c r="L18" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="M18" s="29">
+      <c r="M18" s="26">
         <v>2026</v>
       </c>
-      <c r="N18" s="18" t="s">
+      <c r="N18" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="O18" s="17" t="s">
+      <c r="O18" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="P18" s="33" t="s">
+      <c r="P18" s="28" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="65" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="31" t="s">
+      <c r="F19" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="G19" s="30">
+      <c r="G19" s="32">
         <v>1300000</v>
       </c>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="J19" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="K19" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="M19" s="29">
+      <c r="M19" s="26">
         <v>2026</v>
       </c>
-      <c r="N19" s="23" t="s">
+      <c r="N19" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O19" s="31" t="s">
+      <c r="O19" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="20" t="s">
+      <c r="P19" s="19" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F20" s="31" t="s">
+      <c r="F20" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="G20" s="30">
+      <c r="G20" s="32">
         <v>5500000</v>
       </c>
-      <c r="H20" s="28" t="s">
+      <c r="H20" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="J20" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="K20" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="L20" s="10" t="s">
+      <c r="L20" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="M20" s="29">
+      <c r="M20" s="26">
         <v>2025</v>
       </c>
-      <c r="N20" s="18" t="s">
+      <c r="N20" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="O20" s="31" t="s">
+      <c r="O20" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="P20" s="20" t="s">
+      <c r="P20" s="19" t="s">
         <v>136</v>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
   </sortState>
   <hyperlinks>
     <hyperlink ref="O2" r:id="rId1" xr:uid="{E304E6F9-F947-4494-A94B-6EFAA6BFB69B}"/>
-    <hyperlink ref="O14" r:id="rId2" xr:uid="{91AA9401-501E-4CE7-BDB7-F01C6CBB47B0}"/>
+    <hyperlink ref="O13" r:id="rId2" xr:uid="{91AA9401-501E-4CE7-BDB7-F01C6CBB47B0}"/>
     <hyperlink ref="P18" r:id="rId3" xr:uid="{9AB97224-39A4-4B7F-BDA3-C4983BD9D738}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 5 new listings from spreadsheet: 3801 S Logan St, 4601 W 10th Ave, 1656 Zenobia St, 2256 Curtis St, 14760 SW 64th Ave
Pulled photos from each listing's MLS/Recolorado share link since none
existed locally yet. The spreadsheet's HubSpot Form ID column holds a
hosted-form share link rather than a form UUID for these five, so
build-listings.js now renders an "Inquire About This Property" link
for a URL-shaped hubspotFormId instead of trying to embed it. Also
made the property-specs grid and page copy skip beds/baths/sqft/etc.
gracefully for land listings, which have none of those.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listings/property_listings.xlsx
+++ b/listings/property_listings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1b8a2bdd8672135/Documents/website/listings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AA45C1B-2D7A-4FB9-8B49-2C1C3FA6523F}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97F39807-8BF7-44F2-BD36-6E109F88A248}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="174">
   <si>
     <t>listing_id (slug)</t>
   </si>
@@ -183,21 +183,6 @@
     <t>1,721</t>
   </si>
   <si>
-    <t>3784-fenton-street-wheat-ridge</t>
-  </si>
-  <si>
-    <t>1801607</t>
-  </si>
-  <si>
-    <t>3784 Fenton Street</t>
-  </si>
-  <si>
-    <t>Wheat Ridge</t>
-  </si>
-  <si>
-    <t>1,704</t>
-  </si>
-  <si>
     <t>1642-n-lafayette-street-unit-1-denver</t>
   </si>
   <si>
@@ -327,9 +312,6 @@
     <t>Observatory Park</t>
   </si>
   <si>
-    <t>Fenton Homes</t>
-  </si>
-  <si>
     <t>Under Construction</t>
   </si>
   <si>
@@ -363,9 +345,6 @@
     <t>https://share-na2.hsforms.com/1TOjrZAJAQEaNh7NpXTwYMwq3ct6</t>
   </si>
   <si>
-    <t>https://share-na2.hsforms.com/1Q7HaxHCcTliDJ6GrBoRGMQq3ct6</t>
-  </si>
-  <si>
     <t>https://share-na2.hsforms.com/1a6Dv1AObR46XPc9X9QlZyQq3ct6</t>
   </si>
   <si>
@@ -387,9 +366,6 @@
     <t>https://matrix.recolorado.com/matrix/shared/L83pB7NFM4c/5516ClayCourt</t>
   </si>
   <si>
-    <t>https://matrix.recolorado.com/matrix/shared/dSncCW0JM4c/3784FentonStreet</t>
-  </si>
-  <si>
     <t>https://matrix.recolorado.com/matrix/shared/rQTSDz4KM4c/3927W38thAvenue</t>
   </si>
   <si>
@@ -498,20 +474,95 @@
     <t>1392-swan-peter-drive-berthoud</t>
   </si>
   <si>
-    <t>New Construction Single-Family Home in Wheat Ridge featuring 3 bedrooms, 3 bathrooms, a 2-car garage, and exceptional mountain views. For a limited time, the seller will pay one full year of HOA dues. Designed for modern living, this west-facing home is filled with natural light and offers a spacious, functional floor plan. The main level features a dedicated dining area, casual breakfast space, powder room, and open-concept living areas perfect for everyday living and entertaining. Upstairs, all bedrooms include walk-in closets, while the conveniently located second-floor laundry room adds everyday ease. The private third-floor primary suite is a true retreat, complete with a walkout deck showcasing stunning mountain views. Built for low-maintenance living, this brand-new home is ideal for buyers seeking a lock-and-leave lifestyle without sacrificing space or comfort. Located in the heart of Wheat Ridge, just minutes from Highlands, Edgewater, Sloan’s Lake, and only six miles from Downtown Denver, you'll enjoy easy access to parks, trails, local dining, shopping, and the revitalized 39th Avenue corridor. Don't miss this opportunity to own a new construction home in one of Denver's most desirable and connected neighborhoods.</t>
-  </si>
-  <si>
     <t>921 Mt Massive Drive Unit# 23, Bldg 1</t>
   </si>
   <si>
     <t>Mississippi</t>
+  </si>
+  <si>
+    <t>Land</t>
+  </si>
+  <si>
+    <t>3801 S Logan St</t>
+  </si>
+  <si>
+    <t>Englewood</t>
+  </si>
+  <si>
+    <t>Prime redevelopment opportunity in Englewood. Existing house currently on the property, with the seller in the process of completing key pre-development work, offering significant time and cost savings for the next owner. Buyer may benefit from progress already underway on survey, soils, asbestos abatement, demolition, engineering, and architectural planning. Seller is willing to close upon issuance of permits, providing a streamlined path to construction. Building plans are in Supplements. This project can be delivered fully entitled. The 6,403 square foot lot is zoned for a single-family residence and is ideally located near local amenities, schools, and transportation.</t>
+  </si>
+  <si>
+    <t>https://share-na2.hsforms.com/1hC9LODZdTp2S3UcUyGtYewq3ct6</t>
+  </si>
+  <si>
+    <t>https://matrix.recolorado.com/matrix/shared/k8ClwKsKm6c/3801SLoganStreet</t>
+  </si>
+  <si>
+    <t>https://matrix.recolorado.com/matrix/shared/ywCf3fxLm6c/4601W10thAvenue</t>
+  </si>
+  <si>
+    <t>Property and price offer options. Scrape and rebuild like the duplex to the west or renovate to rent or fix and flip! House has been taken care of and is clean and in rent condition inside, the exterior needs a little love. 6,250-square-foot lot in zoned for up to 2 units. Owner occupants easy sweat equity here and an opportunity to renovate to your style and standards. Conveniently located with easy access to downtown Denver, Sloan’s Lake 7 blocks to the north and amazing restaurants, bars, coffee, yoga, and more a short 7 block walk or bike away to get to all that the south side of Sloan’s Lake offers! A great opportunity to own a single-family home and land in an established Denver neighborhood under 350K! This property is sold "As-Is".</t>
+  </si>
+  <si>
+    <t>4601-w-10th-avenue-denver</t>
+  </si>
+  <si>
+    <t>3801-s-logan-steet-denver</t>
+  </si>
+  <si>
+    <t>4601 W 10th Avenue</t>
+  </si>
+  <si>
+    <t>denver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residental </t>
+  </si>
+  <si>
+    <t>1656-Zenobia-street-denver</t>
+  </si>
+  <si>
+    <t>1656 Zenobia Street</t>
+  </si>
+  <si>
+    <t>Tastefully remodeled and thoughtfully updated, this mid-century modern home offers approximately 4,041 finished square feet with five bedrooms, four bathrooms, a dedicated office, and flexible living spaces across three levels. The main level features engineered hardwood flooring, two bedrooms, abundant storage, and a chef’s kitchen with quartz countertops and full-height backsplash, soft-close solid-wood cabinetry, two pantries, a beverage refrigerator, and high-end Bosch appliances including a 36-inch induction range with downdraft ventilation, double ovens, microwave, dishwasher, and large refrigerator. The expansive upper-level primary retreat features vaulted ceilings, space for a sitting or fitness area, dual custom walk-in closets, and a spa-inspired bath with designer finishes, freestanding soaking tub, steam shower with dual shower heads, bidet wiring, and space for stacked laundry. An adjoining skylit loft offers additional flexible space for a reading nook, workout area, or storage. The finished basement includes two additional bedrooms, a spacious family room ideal for games or a home theater, a kitchenette, and a full laundry room with prep and storage space. Additional highlights include a new gas fireplace, designer tile and lighting, updated windows, LED recessed lighting with night-light settings, luxury vinyl plank, and designer Berber carpet. Outside, enjoy a Trex deck, new cedar fencing, sprinkler system, native Colorado landscaping, oversized detached two-car garage with alley access, front driveway storage for a boat or recreational vehicle, and a large storage shed. Major improvements include a new roof, updated electrical panel, high-efficiency HVAC system, and heat-pump water heater. Ideally located near Sloan’s Lake with convenient access to parks, dining, shopping, and downtown Denver.</t>
+  </si>
+  <si>
+    <t>https://matrix.recolorado.com/matrix/shared/bhMvqGGNm6c/1656ZenobiaStreet</t>
+  </si>
+  <si>
+    <t>https://matrix.recolorado.com/matrix/shared/ZyjSX6KPm6c/2256CurtisStreet</t>
+  </si>
+  <si>
+    <t>DEVELOPMENT OPPORTUNITY: 44-unit Multifamily/Condo Development Opportunity. LOCATION: The project is located in the heart of the rapidly developing Arapahoe Square neighborhood, immediately east of the Central Business District and directly south of LoDo. The location features many amenities and is only one block to Great Divide Brewing, three blocks to Snooze, and five blocks to Coors Field and the center of LoDo. Very close proximity to light rail access and the CBD. ENTITLEMENTS: The project will be sold fully entitled and is exempt from mandatory affordable housing. UNIT MIX: Units ranging from 482-1,118 SqFt. have anticipated sales between $450k-$730k. They will be walkable, in close proximity to downtown and near public transit.</t>
+  </si>
+  <si>
+    <t>2256-curtis-street-denver</t>
+  </si>
+  <si>
+    <t>2256 Curtis Street</t>
+  </si>
+  <si>
+    <t>14760-sw-64th-avenue-arvada</t>
+  </si>
+  <si>
+    <t>14760 SW 64th Avenue</t>
+  </si>
+  <si>
+    <t>Arvada</t>
+  </si>
+  <si>
+    <t>Howard Ranch presents an exceptional opportunity to create an exclusive enclave of luxury lakefront homes at 14760 W. 64th Avenue. Thoughtfully envisioned to showcase the property’s beautiful waterfront setting and expansive views, current plans allow for an elegant residential community featuring 14 finished lots, complete with streets, roads, curb and gutter, and utilities. The property has successfully been rezoned from R-6 to R-A, providing a strong foundation for a distinctive development offering privacy, natural beauty, and refined lakeside living. Soils reports, surveys, environmental studies, civil and structural documents, and building plans are available upon request.</t>
+  </si>
+  <si>
+    <t>https://matrix.recolorado.com/matrix/shared/FJHBMLPQm6c/14760SW64thAvenue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -604,17 +655,23 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF33475B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF33475B"/>
-      <name val="Calibri"/>
+      <b/>
+      <sz val="6"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -686,7 +743,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -750,10 +807,7 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -771,17 +825,24 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1095,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.36328125" style="10" bestFit="1" customWidth="1"/>
@@ -1104,7 +1165,7 @@
     <col min="4" max="4" width="38" style="10" customWidth="1"/>
     <col min="5" max="5" width="14" style="10" customWidth="1"/>
     <col min="6" max="6" width="16" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14" style="27" customWidth="1"/>
+    <col min="7" max="7" width="14" style="26" customWidth="1"/>
     <col min="8" max="8" width="16" style="10" customWidth="1"/>
     <col min="9" max="10" width="7" style="10" customWidth="1"/>
     <col min="11" max="11" width="14" style="10" customWidth="1"/>
@@ -1163,12 +1224,12 @@
         <v>13</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B2" s="6">
         <v>7515586</v>
@@ -1177,13 +1238,13 @@
         <v>17</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="G2" s="15">
         <v>359000</v>
@@ -1205,18 +1266,18 @@
         <v>1961</v>
       </c>
       <c r="N2" s="17" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="P2" s="19" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="B3" s="7">
         <v>7631891</v>
@@ -1225,13 +1286,13 @@
         <v>17</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="G3" s="15">
         <v>375000</v>
@@ -1253,18 +1314,18 @@
         <v>1961</v>
       </c>
       <c r="N3" s="17" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="P3" s="19" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="20" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="B4" s="8">
         <v>4298805</v>
@@ -1273,13 +1334,13 @@
         <v>17</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="G4" s="15">
         <v>400000</v>
@@ -1301,13 +1362,13 @@
         <v>1961</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
@@ -1327,7 +1388,7 @@
         <v>19</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G5" s="21">
         <v>550000</v>
@@ -1351,13 +1412,13 @@
         <v>2024</v>
       </c>
       <c r="N5" s="17" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="O5" s="16" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="P5" s="19" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
@@ -1377,7 +1438,7 @@
         <v>19</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G6" s="21">
         <v>570000</v>
@@ -1401,18 +1462,18 @@
         <v>2026</v>
       </c>
       <c r="N6" s="17" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="O6" s="16" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="P6" s="19" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B7" s="7">
         <v>6797131</v>
@@ -1421,13 +1482,13 @@
         <v>17</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G7" s="15">
         <v>590000</v>
@@ -1451,13 +1512,13 @@
         <v>2024</v>
       </c>
       <c r="N7" s="17" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="O7" s="16" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="P7" s="19" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
@@ -1477,13 +1538,13 @@
         <v>19</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G8" s="21">
-        <v>590000</v>
+        <v>540000</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>21</v>
@@ -1501,33 +1562,33 @@
         <v>2026</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="O8" s="16" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="P8" s="19" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G9" s="21">
         <v>595000</v>
@@ -1542,7 +1603,7 @@
         <v>27</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>23</v>
@@ -1551,13 +1612,13 @@
         <v>2024</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="O9" s="16" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="P9" s="19" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
@@ -1577,13 +1638,13 @@
         <v>19</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G10" s="21">
         <v>625000</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>21</v>
@@ -1601,33 +1662,33 @@
         <v>2026</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="O10" s="16" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="P10" s="19" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="78" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G11" s="21">
         <v>640000</v>
@@ -1642,7 +1703,7 @@
         <v>27</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>23</v>
@@ -1651,13 +1712,13 @@
         <v>2024</v>
       </c>
       <c r="N11" s="22" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="O11" s="16" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="P11" s="19" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
@@ -1677,7 +1738,7 @@
         <v>19</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G12" s="21">
         <v>685000</v>
@@ -1701,18 +1762,18 @@
         <v>2026</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="O12" s="16" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="P12" s="19" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="52" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="B13" s="9">
         <v>9547484</v>
@@ -1721,13 +1782,13 @@
         <v>36</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="G13" s="21">
         <v>699000</v>
@@ -1751,148 +1812,148 @@
         <v>2023</v>
       </c>
       <c r="N13" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="O13" s="29" t="s">
-        <v>108</v>
+        <v>124</v>
+      </c>
+      <c r="O13" s="28" t="s">
+        <v>102</v>
       </c>
       <c r="P13" s="19" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="52" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="G14" s="21">
-        <v>715000</v>
+        <v>830000</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M14" s="16">
         <v>2026</v>
       </c>
-      <c r="N14" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="O14" s="30" t="s">
-        <v>109</v>
+      <c r="N14" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="O14" s="32" t="s">
+        <v>98</v>
       </c>
       <c r="P14" s="19" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>73</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="G15" s="21">
-        <v>830000</v>
+        <v>850000</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M15" s="16">
         <v>2026</v>
       </c>
       <c r="N15" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="O15" s="33" t="s">
-        <v>104</v>
+        <v>126</v>
+      </c>
+      <c r="O15" s="23" t="s">
+        <v>98</v>
       </c>
       <c r="P15" s="19" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="65" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="G16" s="21">
-        <v>850000</v>
+        <v>1000000</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I16" s="9" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="L16" s="9" t="s">
         <v>21</v>
@@ -1900,227 +1961,384 @@
       <c r="M16" s="16">
         <v>2026</v>
       </c>
-      <c r="N16" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="O16" s="24" t="s">
+      <c r="N16" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="P16" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="30">
+        <v>6600690</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="31">
+        <v>1300000</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="I17" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="J17" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="K17" s="30">
+        <v>4013</v>
+      </c>
+      <c r="L17" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="M17" s="25">
+        <v>2026</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="O17" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="P17" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="65" x14ac:dyDescent="0.35">
+      <c r="A18" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="G18" s="31">
+        <v>1300000</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="I18" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="J18" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="K18" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="L18" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" s="25">
+        <v>2026</v>
+      </c>
+      <c r="N18" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="O18" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="P18" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="19" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="65" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A19" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="C19" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="E19" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="31">
+        <v>5500000</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="J19" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="K19" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="L19" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="25">
+        <v>2025</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="O19" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="P19" s="19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="33">
+        <v>7317770</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="G20" s="26">
+        <v>330000</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="N20" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="O20" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="P20" s="27" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A21" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B21" s="34">
+        <v>6307233</v>
+      </c>
+      <c r="C21" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="D21" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="G21" s="26">
+        <v>330000</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" s="10">
+        <v>2</v>
+      </c>
+      <c r="J21" s="10">
+        <v>1</v>
+      </c>
+      <c r="K21" s="10">
+        <v>848</v>
+      </c>
+      <c r="M21" s="10">
+        <v>1951</v>
+      </c>
+      <c r="N21" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="O21" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="P21" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="34">
+        <v>5313629</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="G17" s="21">
-        <v>1000000</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="L17" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="M17" s="16">
-        <v>2026</v>
-      </c>
-      <c r="N17" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="O17" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="P17" s="19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="B18" s="31">
-        <v>6600690</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="31" t="s">
+      <c r="F22" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="G22" s="26">
+        <v>1525000</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I22" s="10">
+        <v>5</v>
+      </c>
+      <c r="J22" s="10">
+        <v>4</v>
+      </c>
+      <c r="K22" s="10">
+        <v>4014</v>
+      </c>
+      <c r="L22" s="10">
+        <v>2</v>
+      </c>
+      <c r="M22" s="10">
+        <v>1953</v>
+      </c>
+      <c r="N22" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="O22" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="G18" s="32">
-        <v>1300000</v>
-      </c>
-      <c r="H18" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="I18" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="J18" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="K18" s="31">
-        <v>4013</v>
-      </c>
-      <c r="L18" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="M18" s="26">
-        <v>2026</v>
-      </c>
-      <c r="N18" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="O18" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="P18" s="28" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="65" x14ac:dyDescent="0.35">
-      <c r="A19" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="F19" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="G19" s="32">
-        <v>1300000</v>
-      </c>
-      <c r="H19" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="I19" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="J19" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="K19" s="31" t="s">
-        <v>33</v>
-      </c>
-      <c r="L19" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="M19" s="26">
-        <v>2026</v>
-      </c>
-      <c r="N19" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="O19" s="30" t="s">
-        <v>106</v>
-      </c>
-      <c r="P19" s="19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A20" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B20" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="G20" s="32">
-        <v>5500000</v>
-      </c>
-      <c r="H20" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="I20" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="J20" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="K20" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="L20" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="M20" s="26">
-        <v>2025</v>
-      </c>
-      <c r="N20" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="O20" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="P20" s="19" t="s">
-        <v>136</v>
-      </c>
+      <c r="P22" s="10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="33">
+        <v>2031493</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="G23" s="26">
+        <v>3200000</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="N23" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="O23" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="P23" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="15" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B24" s="34">
+        <v>3886638</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="G24" s="26">
+        <v>4750000</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="N24" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="O24" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="P24" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="N25" s="35"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P20">
-    <sortCondition ref="G2:G20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P19">
+    <sortCondition ref="G2:G19"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="O2" r:id="rId1" xr:uid="{E304E6F9-F947-4494-A94B-6EFAA6BFB69B}"/>
     <hyperlink ref="O13" r:id="rId2" xr:uid="{91AA9401-501E-4CE7-BDB7-F01C6CBB47B0}"/>
-    <hyperlink ref="P18" r:id="rId3" xr:uid="{9AB97224-39A4-4B7F-BDA3-C4983BD9D738}"/>
+    <hyperlink ref="P17" r:id="rId3" xr:uid="{9AB97224-39A4-4B7F-BDA3-C4983BD9D738}"/>
+    <hyperlink ref="P20" r:id="rId4" xr:uid="{01AB637F-433A-4B5C-9A77-56B1D91452A4}"/>
+    <hyperlink ref="O24" r:id="rId5" xr:uid="{F44CA895-3986-44DB-8048-8F077A924E56}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" r:id="rId4"/>
+  <pageSetup orientation="landscape" r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -2135,10 +2353,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2146,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2154,7 +2372,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2162,7 +2380,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2170,7 +2388,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="28" x14ac:dyDescent="0.35">
@@ -2178,7 +2396,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="28" x14ac:dyDescent="0.35">
@@ -2186,7 +2404,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -2194,15 +2412,15 @@
         <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -2210,7 +2428,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -2218,7 +2436,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update listing descriptions from spreadsheet; reprice 1121 S Dahlia St
Replace generic community blurbs with unit-specific descriptions for
the four Thirty Eight West units and both Birch Leaf duplexes, and
add LEED Platinum mention to 1121 S Dahlia St. Also sync 1121 S
Dahlia St's price to the $675,000 already reflected in the
spreadsheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listings/property_listings.xlsx
+++ b/listings/property_listings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1b8a2bdd8672135/Documents/website/listings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97F39807-8BF7-44F2-BD36-6E109F88A248}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="13_ncr:1_{D25EC43F-11B6-4128-9ED2-E6F28545FCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{369454D1-7A2A-4F08-B243-DEAD1841357B}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="177">
   <si>
     <t>listing_id (slug)</t>
   </si>
@@ -393,27 +393,12 @@
     <t>https://matrix.recolorado.com/matrix/shared/JY7N7GztN4c/1652NLafayetteStreet</t>
   </si>
   <si>
-    <t>Embrace a harmonious blend of sustainability and comfort with these three duplexes on Columbine Lane in Denver's thriving metro area. Situated within easy reach of Denver’s exciting downtown, enjoy all of the urban conveniences while having a cozy retreat in a quiet suburban setting to come home to. This eco-conscious half duplex home features Energy Star appliances and is primed to attain LEED Gold certification, promising a greener, healthier lifestyle without sacrificing modern comforts. You’ll love the welcoming open floor plan and revel in the chic allure of the kitchen’s quartz countertops, beautiful soft-close cabinetry, a suite of stainless appliances, and the seamless integration of smart home technology. Your new home offers 3 bedrooms and 2.5 baths (including an ensuite bath in the primary bedroom), and an oversized 2-car garage.</t>
-  </si>
-  <si>
-    <t>Welcome to LiteTowns, a collection of modern new construction townhomes in Denver's highly sought-after City Park West neighborhood. This thoughtfully designed 3-story townhome offers 3 bedrooms, 2.5 bathrooms, and 1,514 square feet of stylish, low-maintenance living in one of Denver's most walkable and vibrant locations. Inside, you'll find an open-concept floor plan filled with natural light, contemporary finishes, and functional living spaces designed for today's lifestyle. The gourmet kitchen features quartz countertops, soft-close cabinetry, stainless steel appliances, and ample storage, creating the perfect space for entertaining and everyday living. An attached 1-car garage adds convenience and secure parking. Built with energy-efficient construction and designed to meet LEED Gold standards, this home offers lower utility costs, improved comfort, and sustainable living without compromising style. Ideally located near City Park, Cheesman Park, the Denver Botanic Gardens, Denver Zoo, Denver Museum of Nature &amp; Science, and City Park Golf Course, residents enjoy easy access to some of Denver's most iconic destinations. Walk to neighborhood restaurants, coffee shops, breweries, and shopping while enjoying quick access to Downtown Denver, Cherry Creek, and major commuter routes. Whether you're seeking a primary residence, lock-and-leave lifestyle, or low-maintenance urban living, this move-in-ready townhome offers the perfect combination of location, design, and convenience. Property is governed by a Party Wall Agreement. Monthly fee is $113. See supplements for details.</t>
-  </si>
-  <si>
     <t>Welcome to LiteTowns, a collection of modern new construction townhomes in Denver's highly sought-after City Park West neighborhood. This thoughtfully designed 3-story townhome offers 2 bedrooms, 2.5 bathrooms, and 1,448 square feet of stylish, low-maintenance living in one of Denver's most walkable and vibrant locations. Inside, you'll find an open-concept floor plan filled with natural light, contemporary finishes, and functional living spaces designed for today's lifestyle. The gourmet kitchen features quartz countertops, soft-close cabinetry, stainless steel appliances, and ample storage, creating the perfect space for entertaining and everyday living. An attached 1-car garage adds convenience and secure parking. Built with energy-efficient construction and designed to meet LEED Gold standards, this home offers lower utility costs, improved comfort, and sustainable living without compromising style. Ideally located near City Park, Cheesman Park, the Denver Botanic Gardens, Denver Zoo, Denver Museum of Nature &amp; Science, and City Park Golf Course, residents enjoy easy access to some of Denver's most iconic destinations. Walk to neighborhood restaurants, coffee shops, breweries, and shopping while enjoying quick access to Downtown Denver, Cherry Creek, and major commuter routes. Whether you're seeking a primary residence, lock-and-leave lifestyle, or low-maintenance urban living, this move-in-ready townhome offers the perfect combination of location, design, and convenience. Property is governed by a Party Wall Agreement. Monthly fee is $113. See supplements for details.</t>
   </si>
   <si>
-    <t>Welcome to Thirty Eight West, an exciting new construction community featuring 25 thoughtfully designed residences in a prime Denver location. Offering contemporary architecture, functional floor plans, and quality craftsmanship, this highly anticipated development combines modern living with exceptional convenience. Homes are currently priced from the mid-$600,000s to $1.4 million and offer a variety of layouts designed for today's lifestyle. Residents will enjoy open-concept living spaces, designer finishes, abundant natural light, energy-efficient construction, and low-maintenance homeownership. Ideally located near Denver's popular dining, shopping, parks, and entertainment destinations, Thirty Eight West provides easy access to Downtown Denver, major commuter routes, public transit, and outdoor recreation. Whether you're looking for a primary residence, a lock-and-leave lifestyle, or a brand-new home in a thriving neighborhood, Thirty Eight West offers the perfect blend of style, comfort, and location. With anticipated deliveries beginning Summer–Fall 2026, now is the opportunity to secure a home in one of Denver's newest communities before completion. This community will be governed by a Party Wall Agreement. Management fees are currently being finalized and are subject to change.</t>
-  </si>
-  <si>
     <t>Welcome to LiteTowns, a collection of modern new construction townhomes in Denver's highly sought-after City Park West neighborhood. This desirable end-unit townhome offers 2 bedrooms, 2.5 bathrooms, and 1,642 square feet of stylish, low-maintenance living in one of Denver's most walkable and vibrant locations. Inside, you'll find an open-concept floor plan filled with natural light, contemporary finishes, and functional living spaces designed for today's lifestyle. The gourmet kitchen features quartz countertops, soft-close cabinetry, stainless steel appliances, and ample storage, creating the perfect space for entertaining and everyday living. As an end unit, this home benefits from additional windows, enhanced privacy, and abundant natural light throughout. An attached 1-car garage adds convenience and secure parking. Built with energy-efficient construction and designed to meet LEED Gold standards, this home offers lower utility costs, improved comfort, and sustainable living without compromising style. Ideally located near City Park, Cheesman Park, the Denver Botanic Gardens, Denver Zoo, Denver Museum of Nature &amp; Science, and City Park Golf Course, residents enjoy easy access to some of Denver's most iconic destinations. Walk to neighborhood restaurants, coffee shops, breweries, and shopping while enjoying quick access to Downtown Denver, Cherry Creek, and major commuter routes. Whether you're seeking a primary residence, lock-and-leave lifestyle, or low-maintenance urban living, this move-in-ready townhome offers the perfect combination of location, design, and convenience. Property is governed by a Party Wall Agreement. Monthly fee is $113. See supplements for details.</t>
   </si>
   <si>
-    <t>The Future is Now! Discover what it means to fully embrace a sustainable lifestyle. The LiteHomes at Mississippi offer a sleek modern concept, with simple clean lines and finishes inside and out. Everything was taken into consideration for this design, from lot orientation to floor plan flow and elevation, to window placement to make the most of the available natural light and resources. The creative and thoughtfully designed split-level floor plan features a Scandinavian-inspired, open-concept layout with the upper level boasting a welcoming living room, gorgeous kitchen, bright dining area and a half bath. Alternatively, the bedrooms are conveniently nestled in the restful and private lower level. With four bedrooms and three bathrooms, this home offers ample space for comfortable, healthy, sustainable, living. And just wait until you see the primary suite! These homes also offer a welcoming back yard and detached, single-car garage. Enjoy the convenience of being close to the desirable Cherry Creek neighborhood amenities, where you'll find an extended array of shopping, dining, and entertainment options. Experience this state-of-the-art home's perfect harmony of sustainability, efficiency, style, and location.</t>
-  </si>
-  <si>
-    <t>Welcome to Birch Leaf, an exclusive collection of five modern duplex residences by redT Homes. These thoughtfully designed new construction homes offer 3–4 bedrooms, approximately 1,681–2,000 square feet, open-concept floor plans, abundant natural light, and designer-selected finishes. Conveniently located near Regis University with easy access to shopping, dining, parks, and major commuter routes, Birch Leaf combines modern living with exceptional convenience. Quality craftsmanship, contemporary design, and functional living spaces make these homes ideal for today's lifestyle. This is an active construction site. All visitors must be accompanied by an agent or representative and wear appropriate safety gear, including hard hats and closed-toe shoes. Property is governed by a Party Wall Agreement and managed by Royal Oak Property Management. Monthly assessments are currently being finalized and are subject to change. Being respectful of Colorado's drought conditions to not water grass while no one is home. City will grant a water establishment permit and we will schedule grass install upon contract. This property is governed by a party wall agreement and managed by Royal Oak Property Management. Monthly assessment information TBD.</t>
-  </si>
-  <si>
     <t>Modern new construction featuring a third floor is dedicated to an additional primary suite with a large bath, walk-in closet, and access to a private rooftop deck. Thoughtful finishes are featured throughout, including a stainless steel appliance package with range, over-the-range microwave, full-size refrigerator, and dishwasher, an undermount stainless steel kitchen sink, quartz countertops and backsplash, solid wood soft-close shaker cabinetry in a light wood finish, LVP flooring throughout the main living areas, tile in all bathrooms, Berber carpet in the bedrooms, and a private yard. This 3-bedroom, 3.5-bath layout offers a rare three-primary-suite design at this price point. The open main level features a spacious living area and convenient powder bath. The second floor includes two primary bedrooms, each with walk-in closets and en-suite baths. A one-car detached garage completes the package. Located in Rosedale, walkable to Platt Park and Harvard Gulch, with a Walk Score of 88 and no HOA.</t>
   </si>
   <si>
@@ -556,6 +541,30 @@
   </si>
   <si>
     <t>https://matrix.recolorado.com/matrix/shared/FJHBMLPQm6c/14760SW64thAvenue</t>
+  </si>
+  <si>
+    <t>Embrace a harmonious blend of sustainability and comfort with these three duplexes on Columbine Lane in Denver's thriving metro area. Situated within easy reach of Denver’s exciting downtown, enjoy all of the urban conveniences while having a cozy retreat in a quiet suburban setting to come home to. This eco-conscious half duplex home features Energy Star appliances and is primed to attain LEED Gold certification, promising a greener, healthier lifestyle without sacrificing modern comforts. You’ll love the welcoming open floor plan and revel in the chic allure of the kitchen’s quartz countertops, beautiful soft-close cabinetry, a suite of stainless appliances, and the seamless integration of smart home technology. Your new home offers 3 bedrooms and 2.5 baths (including an ensuite bath in the primary bedroom), and an oversized 2-car garage</t>
+  </si>
+  <si>
+    <t>A true lock-off suite on the main floor with its own bedroom, full bath, and full kitchen, and it can be completely closed off from the rest of the house if the buyer chooses. That flexibility is almost impossible to find in new construction in the Highlands, and it's what makes this the most interesting floor plan at Thirty Eight West. At 3,011 square feet, this is the largest home in the community: five bedrooms, five full baths, and two complete kitchens. Upstairs holds the primary suite, three more bedrooms, a second kitchen, and a second living and dining area so the two halves of the home genuinely function on their own. Multigenerational households, a live-in guest suite, Airbnb, separate long term rental, or anyone who needs real separation of space, the house hacking opportunities are endless in this home. Very large Rooftop deck with mountain views and private patios. In-unit laundry, quartz counters, a five-piece primary bath, wood, tile, and carpet flooring, forced-air heat, central air, attached garage. No HOA dues; a party wall agreement governs shared elements. Walk Score 93 with Tennyson Street, Highlands Square, and two neighborhood parks all within walking distance. This unit is essentially complete and awaiting appliances, with delivery expected within 30 days. Permanent rate buydown available through November with preferred lender partners. Hard hats required until final CO call for a same-day showing with a sales rep 303-353-1574</t>
+  </si>
+  <si>
+    <t>Only one shared wall and a two-car attached garage this Building 6 residence is one of the most private homes at Thirty Eight West, and it's nearly ready. Appliances and a few final installs are all that remain, with delivery expected within 30 days. 1,897 finished square feet across three levels. Three bedrooms and three full baths sit together on the upper level alongside the open living, dining, and kitchen space, plus a flexible loft that works as an office, den, or guest room. The main level keeps a powder room and a dedicated laundry room out of the way of daily living. Quartz counters, a five-piece primary bath, wood, tile, and carpet flooring, ceiling fans, high-speed internet ready, forced-air heat, and central air. No HOA dues shared elements are governed by a party wall agreement, so you keep the low-maintenance benefits without the monthly bill. Walk Score 93 puts Tennyson Street's restaurants and shops, Highlands Square, and Berkeley and Rocky Mountain Lake Parks within easy reach, with a quick drive to downtown Denver and I-70 west to the mountains. Permanent rate buydown available through November with the builder's preferred lender partners. Hard hats required until final CO same-day showings available with a sales representative, just call ahead.</t>
+  </si>
+  <si>
+    <t>The largest home at Birch Leaf, on the end, with a two-car attached garage. 1,979 square feet, nearly 300 more than its neighbor, at $346 per square foot. As an end unit with only one shared wall, this home gets windows on three sides. The main level runs living room to dining to kitchen, with a powder bath and a dedicated main-floor office. A real door to close, not a corner of the living room. Upstairs holds three bedrooms including a primary with an en-suite three-quarter bath, a second full bath, and the laundry. Open-concept layout, abundant natural light, designer-selected finishes, forced-air heat, and central air. Two-car attached garage. Crawl space for storage. Birch Leaf is a five-home collection by redT Homes near Regis University, with easy access to shopping, dining, parks, and I-70 and I-76. NO HOA!! A party wall agreement covers the pond and snow removal, managed by Royal Oak Property Management, at roughly $100-$150 monthly. Permanent rate buydown available through November with redT Homes' preferred lender partners, ask for current terms. Grass is installed at closing; the city grants the water establishment permit once a home is under contract, and we schedule the install then. Virtual tour available. Book through ShowingTime or call our sales team directly 303-353-1574</t>
+  </si>
+  <si>
+    <t>The Future is Now! Discover what it means to fully embrace a sustainable lifestyle. This contemporary, energy-efficient, LEED Platinum Certified LiteHome, located at 1121 S Dahlia Street in Denver, is part of a game-changing development. The LiteHomes at Mississippi offer a sleek modern concept with simple, clean lines and finishes inside and out. Everything was taken into consideration for this design, from lot orientation to floor plan flow and elevation, to window placement, to make the most of the available natural light and resources. The creative and thoughtfully designed split-level floor plan features a Scandinavian-inspired, open-concept layout with the upper level boasting a welcoming living room, gorgeous kitchen, bright dining area, and a half bath. Alternatively, the bedrooms are conveniently nestled in the restful and private garden level. With four bedrooms and three bathrooms, this home offers ample space for comfortable, healthy, sustainable living. And just wait until you see the primary suite! These homes also offer a welcoming backyard and detached, single-car garage. Enjoy the convenience of being close to the desirable Cherry Creek neighborhood amenities, where you'll find an extended array of shopping, dining, and entertainment options, all within a three-minute drive. Experience this state-of-the-art home's perfect harmony of sustainability, efficiency, style, and location.</t>
+  </si>
+  <si>
+    <t>Rooftop deck, private patio, two-car garage, and $389 per square foot. 1,605 square feet with three total levels of living space + a large rooftop deck with mountain views. The main level opens with a welcoming and sun filled living room/foyer, the second floor holds the kitchen, a second living area with a deck attached, dining space, a powder room. The next floor up we have two bedrooms that each have their own full bath and are positioned next to the laundry space. It's a layout that works whether you're sharing the home or want a real guest suite instead of a spare room. Quartz counters, a five-piece primary bath, wood, tile, and carpet flooring in the bedrooms, ceiling fans, forced-air heat, and central air. Two car attached garage spaces are hard to come by at this price in 80212. This is the best value at Thirty Eight West, and it's essentially finished. Everything is installed but appliances, with delivery expected within 30 days. Same-day showings available with a sales representative on site. No HOA dues shared elements are governed by a party wall agreement. Walk Score 93. Tennyson Street, Highlands Square, and both Berkeley and Rocky Mountain Lake Parks are an easy walk, with downtown Denver minutes away. Permanent rate buydowns available through November with the builder's preferred lender partners (ask for current terms). Hard hats required until final CO, so call to schedule; we can usually get you in the same day 303-353-1574</t>
+  </si>
+  <si>
+    <t>New construction under $575,000, on the end, with all three bedrooms upstairs. At $339 per square foot, this is the best value at Birch Leaf. 1,681 square feet on two levels. The main floor opens across a separate dining room and living room, with a powder bath tucked out of the way. Upstairs holds all three bedrooms, including a primary with an en-suite three-quarter bath, plus a second full bath and the laundry room and no hauling baskets between floors. Only one shared wall, so windows on three sides. Open-concept design, abundant natural light, designer-selected finishes, forced-air heat, and central air. Attached one-car garage plus a crawl space for storage. Birch Leaf is a five-home collection by redT Homes near Regis University, close to shopping, dining, parks, and the I-70 and I-76 corridors. NO HOA!!! A party wall agreement covers the pond and snow removal and should be roughly $100-$150 monthly. Permanent rate buydown available through November with redT Homes' preferred lender partners (ask for current terms). Grass is installed at closing once the city grants the water establishment permit. Schedule a showing through ShowingTime or reach out to our sales team directly at 303-353-1574</t>
+  </si>
+  <si>
+    <t>Brand-new construction in the Highlands under $550,000 is the most attainable home at Thirty Eight West, and it delivers in weeks, not months. Building 5 is at drywall with completion expected in the next 30 days or less. 1,168 square feet across three levels with a private attached garage. The main-level foyer opens the home up and can be used for a living room, mud room, or office space, while the kitchen, main living room, first bedroom and full bathroom are one floor up. On the top floor we have another full bedroom and bathroom next to a bonus loft that works as a home office, gym, or reading nook. Both bedrooms are on the upper levels, each served by a full bath. This home features quartz counters, two large bathrooms and bedrooms, ceiling fans, forced-air heat, central air, and a smoke-free build throughout. This home is very private and quiet with no noise pollution. No HOA dues and a party wall agreement governs shared elements, so there's no monthly association bill. Walk Score 93. Tennyson Street, Highlands Square, and two neighborhood parks are within walking distance, with quick access to I-70, downtown Denver, and the mountains. Permanent rate buydown available through November with the builder's preferred lender partners. On a home at this price, that's real monthly savings worth running the numbers on!! Hard hats required until final CO; same-day showings available with a sales representative on site. Please call 303-353-1574 for more information and showings!</t>
   </si>
 </sst>
 </file>
@@ -743,7 +752,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -804,9 +813,6 @@
     <xf numFmtId="4" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -832,9 +838,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -843,6 +846,28 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1165,7 +1190,7 @@
     <col min="4" max="4" width="38" style="10" customWidth="1"/>
     <col min="5" max="5" width="14" style="10" customWidth="1"/>
     <col min="6" max="6" width="16" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14" style="26" customWidth="1"/>
+    <col min="7" max="7" width="14" style="25" customWidth="1"/>
     <col min="8" max="8" width="16" style="10" customWidth="1"/>
     <col min="9" max="10" width="7" style="10" customWidth="1"/>
     <col min="11" max="11" width="14" style="10" customWidth="1"/>
@@ -1228,122 +1253,114 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="B2" s="6">
+      <c r="A2" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" s="36">
+        <v>7317770</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="G2" s="40">
+        <v>330000</v>
+      </c>
+      <c r="H2" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="O2" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="P2" s="19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A3" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="37">
+        <v>6307233</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="40">
+        <v>330000</v>
+      </c>
+      <c r="H3" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="34">
+        <v>2</v>
+      </c>
+      <c r="J3" s="34">
+        <v>1</v>
+      </c>
+      <c r="K3" s="34">
+        <v>848</v>
+      </c>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34">
+        <v>1951</v>
+      </c>
+      <c r="N3" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="O3" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="P3" s="19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="6">
         <v>7515586</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="15">
-        <v>359000</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="8">
-        <v>2</v>
-      </c>
-      <c r="J2" s="8">
-        <v>1</v>
-      </c>
-      <c r="K2" s="8">
-        <v>896</v>
-      </c>
-      <c r="L2" s="8"/>
-      <c r="M2" s="16">
-        <v>1961</v>
-      </c>
-      <c r="N2" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="P2" s="19" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="B3" s="7">
-        <v>7631891</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="G3" s="15">
-        <v>375000</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="8">
-        <v>2</v>
-      </c>
-      <c r="J3" s="8">
-        <v>1</v>
-      </c>
-      <c r="K3" s="8">
-        <v>896</v>
-      </c>
-      <c r="L3" s="8"/>
-      <c r="M3" s="16">
-        <v>1961</v>
-      </c>
-      <c r="N3" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="P3" s="19" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="B4" s="8">
-        <v>4298805</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>146</v>
+      <c r="D4" s="9" t="s">
+        <v>124</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="G4" s="15">
-        <v>400000</v>
+        <v>359000</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>20</v>
@@ -1362,110 +1379,106 @@
         <v>1961</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="O4" s="8" t="s">
-        <v>137</v>
+        <v>126</v>
+      </c>
+      <c r="O4" s="18" t="s">
+        <v>132</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>44</v>
+        <v>128</v>
+      </c>
+      <c r="B5" s="7">
+        <v>7631891</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="G5" s="21">
-        <v>550000</v>
+        <v>125</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="G5" s="15">
+        <v>375000</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>21</v>
-      </c>
+      <c r="I5" s="8">
+        <v>2</v>
+      </c>
+      <c r="J5" s="8">
+        <v>1</v>
+      </c>
+      <c r="K5" s="8">
+        <v>896</v>
+      </c>
+      <c r="L5" s="8"/>
       <c r="M5" s="16">
-        <v>2024</v>
+        <v>1961</v>
       </c>
       <c r="N5" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="O5" s="16" t="s">
-        <v>96</v>
+        <v>127</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>132</v>
       </c>
       <c r="P5" s="19" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>35</v>
+      <c r="A6" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4298805</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>37</v>
+        <v>17</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>141</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G6" s="21">
-        <v>570000</v>
+        <v>125</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="G6" s="15">
+        <v>400000</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>23</v>
-      </c>
+      <c r="I6" s="8">
+        <v>2</v>
+      </c>
+      <c r="J6" s="8">
+        <v>1</v>
+      </c>
+      <c r="K6" s="8">
+        <v>896</v>
+      </c>
+      <c r="L6" s="8"/>
       <c r="M6" s="16">
-        <v>2026</v>
+        <v>1961</v>
       </c>
       <c r="N6" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="O6" s="16" t="s">
-        <v>101</v>
+        <v>130</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>132</v>
       </c>
       <c r="P6" s="19" t="s">
         <v>113</v>
@@ -1473,49 +1486,49 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" s="7">
-        <v>6797131</v>
+        <v>15</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>116</v>
+      <c r="D7" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" s="15">
-        <v>590000</v>
+        <v>88</v>
+      </c>
+      <c r="G7" s="21">
+        <v>540000</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="8">
-        <v>3</v>
-      </c>
-      <c r="J7" s="8">
-        <v>3</v>
-      </c>
-      <c r="K7" s="8">
-        <v>1514</v>
-      </c>
-      <c r="L7" s="8">
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M7" s="16">
-        <v>2024</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>120</v>
+        <v>2026</v>
+      </c>
+      <c r="N7" s="31" t="s">
+        <v>176</v>
       </c>
       <c r="O7" s="16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="P7" s="19" t="s">
         <v>118</v>
@@ -1523,49 +1536,49 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G8" s="21">
-        <v>540000</v>
+        <v>550000</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="I8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="L8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>23</v>
-      </c>
       <c r="M8" s="16">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>122</v>
+        <v>169</v>
       </c>
       <c r="O8" s="16" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="P8" s="19" t="s">
         <v>112</v>
@@ -1573,49 +1586,49 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G9" s="21">
-        <v>595000</v>
+        <v>570000</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>20</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>23</v>
       </c>
       <c r="M9" s="16">
-        <v>2024</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>121</v>
+        <v>2026</v>
+      </c>
+      <c r="N9" s="31" t="s">
+        <v>175</v>
       </c>
       <c r="O9" s="16" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P9" s="19" t="s">
         <v>114</v>
@@ -1623,66 +1636,66 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>25</v>
+        <v>117</v>
+      </c>
+      <c r="B10" s="7">
+        <v>6797131</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>26</v>
+      <c r="D10" s="20" t="s">
+        <v>116</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="G10" s="21">
-        <v>625000</v>
+        <v>95</v>
+      </c>
+      <c r="G10" s="15">
+        <v>590000</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="I10" s="8">
+        <v>3</v>
+      </c>
+      <c r="J10" s="8">
+        <v>3</v>
+      </c>
+      <c r="K10" s="8">
+        <v>1514</v>
+      </c>
+      <c r="L10" s="8">
+        <v>1</v>
       </c>
       <c r="M10" s="16">
-        <v>2026</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>122</v>
+        <v>2024</v>
+      </c>
+      <c r="N10" s="31" t="s">
+        <v>119</v>
       </c>
       <c r="O10" s="16" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P10" s="19" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="78" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>19</v>
@@ -1691,7 +1704,7 @@
         <v>95</v>
       </c>
       <c r="G11" s="21">
-        <v>640000</v>
+        <v>595000</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1703,7 +1716,7 @@
         <v>27</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>23</v>
@@ -1711,8 +1724,8 @@
       <c r="M11" s="16">
         <v>2024</v>
       </c>
-      <c r="N11" s="22" t="s">
-        <v>123</v>
+      <c r="N11" s="31" t="s">
+        <v>119</v>
       </c>
       <c r="O11" s="16" t="s">
         <v>103</v>
@@ -1723,37 +1736,37 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="G12" s="21">
-        <v>685000</v>
+        <v>625000</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>21</v>
@@ -1761,111 +1774,111 @@
       <c r="M12" s="16">
         <v>2026</v>
       </c>
-      <c r="N12" s="17" t="s">
-        <v>125</v>
+      <c r="N12" s="31" t="s">
+        <v>174</v>
       </c>
       <c r="O12" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P12" s="19" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="52" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="B13" s="9">
-        <v>9547484</v>
+        <v>49</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>139</v>
+        <v>51</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>147</v>
+        <v>95</v>
       </c>
       <c r="G13" s="21">
-        <v>699000</v>
+        <v>640000</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M13" s="16">
-        <v>2023</v>
-      </c>
-      <c r="N13" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="O13" s="28" t="s">
-        <v>102</v>
+        <v>2024</v>
+      </c>
+      <c r="N13" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="O13" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="P13" s="19" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G14" s="21">
-        <v>830000</v>
+        <v>685000</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M14" s="16">
         <v>2026</v>
       </c>
-      <c r="N14" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="O14" s="32" t="s">
-        <v>98</v>
+      <c r="N14" s="31" t="s">
+        <v>172</v>
+      </c>
+      <c r="O14" s="39" t="s">
+        <v>101</v>
       </c>
       <c r="P14" s="19" t="s">
         <v>108</v>
@@ -1873,75 +1886,75 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>72</v>
+        <v>135</v>
+      </c>
+      <c r="B15" s="9">
+        <v>9547484</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>73</v>
+        <v>134</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>89</v>
+        <v>142</v>
       </c>
       <c r="G15" s="21">
-        <v>850000</v>
+        <v>675000</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>27</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>21</v>
       </c>
       <c r="M15" s="16">
-        <v>2026</v>
-      </c>
-      <c r="N15" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="O15" s="23" t="s">
-        <v>98</v>
+        <v>2023</v>
+      </c>
+      <c r="N15" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="O15" s="27" t="s">
+        <v>102</v>
       </c>
       <c r="P15" s="19" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="65" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G16" s="21">
-        <v>1000000</v>
+        <v>830000</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>92</v>
@@ -1953,19 +1966,19 @@
         <v>47</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M16" s="16">
         <v>2026</v>
       </c>
-      <c r="N16" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="O16" s="16" t="s">
-        <v>100</v>
+      <c r="N16" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="O16" s="22" t="s">
+        <v>98</v>
       </c>
       <c r="P16" s="19" t="s">
         <v>106</v>
@@ -1973,98 +1986,98 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="B17" s="30">
-        <v>6600690</v>
-      </c>
-      <c r="C17" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="F17" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="31">
-        <v>1300000</v>
-      </c>
-      <c r="H17" s="24" t="s">
+      <c r="D17" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="41">
+        <v>850000</v>
+      </c>
+      <c r="H17" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="I17" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="J17" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="K17" s="30">
-        <v>4013</v>
-      </c>
-      <c r="L17" s="30" t="s">
+      <c r="I17" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="K17" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="L17" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="24">
+        <v>2026</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="O17" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="P17" s="26" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A18" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="G18" s="41">
+        <v>1000000</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I18" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="M17" s="25">
+      <c r="K18" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="L18" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="M18" s="24">
         <v>2026</v>
       </c>
-      <c r="N17" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="O17" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="P17" s="27" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="65" x14ac:dyDescent="0.35">
-      <c r="A18" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="G18" s="31">
-        <v>1300000</v>
-      </c>
-      <c r="H18" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="I18" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="J18" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="K18" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="L18" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" s="25">
-        <v>2026</v>
-      </c>
-      <c r="N18" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="O18" s="29" t="s">
+      <c r="N18" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="O18" s="39" t="s">
         <v>100</v>
       </c>
       <c r="P18" s="19" t="s">
@@ -2072,270 +2085,288 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A19" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" s="24" t="s">
+      <c r="A19" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="29">
+        <v>6600690</v>
+      </c>
+      <c r="C19" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="24" t="s">
+      <c r="D19" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="G19" s="30">
+        <v>1300000</v>
+      </c>
+      <c r="H19" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I19" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="J19" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="K19" s="29">
+        <v>4013</v>
+      </c>
+      <c r="L19" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="M19" s="24">
+        <v>2026</v>
+      </c>
+      <c r="N19" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="O19" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="P19" s="19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A20" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" s="31">
-        <v>5500000</v>
-      </c>
-      <c r="H19" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="J19" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="K19" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="L19" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="M19" s="25">
-        <v>2025</v>
-      </c>
-      <c r="N19" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="O19" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="P19" s="19" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="B20" s="33">
-        <v>7317770</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="F20" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="30">
+        <v>1300000</v>
+      </c>
+      <c r="H20" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="I20" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="J20" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="K20" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="L20" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="M20" s="39">
+        <v>2026</v>
+      </c>
+      <c r="N20" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="O20" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="P20" s="26" t="s">
         <v>148</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="G20" s="26">
-        <v>330000</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="N20" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="O20" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="P20" s="27" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B21" s="34">
-        <v>6307233</v>
-      </c>
-      <c r="C21" s="24" t="s">
+      <c r="B21" s="32">
+        <v>5313629</v>
+      </c>
+      <c r="C21" s="38" t="s">
         <v>36</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>159</v>
+        <v>19</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="G21" s="26">
-        <v>330000</v>
+        <v>155</v>
+      </c>
+      <c r="G21" s="25">
+        <v>1525000</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>20</v>
       </c>
       <c r="I21" s="10">
+        <v>5</v>
+      </c>
+      <c r="J21" s="10">
+        <v>4</v>
+      </c>
+      <c r="K21" s="10">
+        <v>4014</v>
+      </c>
+      <c r="L21" s="10">
         <v>2</v>
       </c>
-      <c r="J21" s="10">
-        <v>1</v>
-      </c>
-      <c r="K21" s="10">
-        <v>848</v>
-      </c>
       <c r="M21" s="10">
-        <v>1951</v>
-      </c>
-      <c r="N21" s="33" t="s">
-        <v>155</v>
+        <v>1953</v>
+      </c>
+      <c r="N21" s="31" t="s">
+        <v>158</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B22" s="31">
+        <v>2031493</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G22" s="25">
+        <v>3200000</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="N22" s="31" t="s">
         <v>161</v>
       </c>
-      <c r="B22" s="34">
-        <v>5313629</v>
-      </c>
-      <c r="C22" s="10" t="s">
+      <c r="O22" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="P22" s="10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="15" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23" s="32">
+        <v>3886638</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G23" s="25">
+        <v>4750000</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="N23" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="O23" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="P23" s="10" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A24" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="E22" s="10" t="s">
+      <c r="D24" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="G22" s="26">
-        <v>1525000</v>
-      </c>
-      <c r="H22" s="10" t="s">
+      <c r="F24" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" s="30">
+        <v>5500000</v>
+      </c>
+      <c r="H24" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="I22" s="10">
-        <v>5</v>
-      </c>
-      <c r="J22" s="10">
-        <v>4</v>
-      </c>
-      <c r="K22" s="10">
-        <v>4014</v>
-      </c>
-      <c r="L22" s="10">
-        <v>2</v>
-      </c>
-      <c r="M22" s="10">
-        <v>1953</v>
-      </c>
-      <c r="N22" s="33" t="s">
-        <v>163</v>
-      </c>
-      <c r="O22" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="P22" s="10" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="B23" s="33">
-        <v>2031493</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="D23" s="10" t="s">
+      <c r="I24" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="J24" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="K24" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="M24" s="39">
+        <v>2025</v>
+      </c>
+      <c r="N24" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="O24" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="P24" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="F23" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="G23" s="26">
-        <v>3200000</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="N23" s="33" t="s">
-        <v>166</v>
-      </c>
-      <c r="O23" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="P23" s="10" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="15" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="B24" s="34">
-        <v>3886638</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="G24" s="26">
-        <v>4750000</v>
-      </c>
-      <c r="H24" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="N24" s="34" t="s">
-        <v>172</v>
-      </c>
-      <c r="O24" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="P24" s="10" t="s">
-        <v>173</v>
-      </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="N25" s="35"/>
+      <c r="N25" s="33"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P19">
-    <sortCondition ref="G2:G19"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O24">
+    <sortCondition ref="G2:G24"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="O2" r:id="rId1" xr:uid="{E304E6F9-F947-4494-A94B-6EFAA6BFB69B}"/>
-    <hyperlink ref="O13" r:id="rId2" xr:uid="{91AA9401-501E-4CE7-BDB7-F01C6CBB47B0}"/>
+    <hyperlink ref="O4" r:id="rId1" xr:uid="{E304E6F9-F947-4494-A94B-6EFAA6BFB69B}"/>
+    <hyperlink ref="O15" r:id="rId2" xr:uid="{91AA9401-501E-4CE7-BDB7-F01C6CBB47B0}"/>
     <hyperlink ref="P17" r:id="rId3" xr:uid="{9AB97224-39A4-4B7F-BDA3-C4983BD9D738}"/>
     <hyperlink ref="P20" r:id="rId4" xr:uid="{01AB637F-433A-4B5C-9A77-56B1D91452A4}"/>
-    <hyperlink ref="O24" r:id="rId5" xr:uid="{F44CA895-3986-44DB-8048-8F077A924E56}"/>
+    <hyperlink ref="O23" r:id="rId5" xr:uid="{F44CA895-3986-44DB-8048-8F077A924E56}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId6"/>

</xml_diff>